<commit_message>
version 1 of analysis
</commit_message>
<xml_diff>
--- a/data/timeline/timeline.xlsx
+++ b/data/timeline/timeline.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/walker/Documents/Github/wind-tunnel-flies/data/timeline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C10C1DA-9935-C547-9A27-49588BA7B3A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A926F2-4879-664B-A799-3B84F7C153CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="640" yWindow="3640" windowWidth="27640" windowHeight="16160" xr2:uid="{935CCC79-5EEF-0F46-B060-FF3944800905}"/>
+    <workbookView xWindow="960" yWindow="1800" windowWidth="27640" windowHeight="16160" xr2:uid="{935CCC79-5EEF-0F46-B060-FF3944800905}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>start date</t>
   </si>
@@ -71,9 +71,6 @@
     <t>Rep B of wing shape data</t>
   </si>
   <si>
-    <t>L45 founded</t>
-  </si>
-  <si>
     <t>Wheeler wind tunnel data</t>
   </si>
   <si>
@@ -87,6 +84,12 @@
   </si>
   <si>
     <t>Weight data for Weber 2006</t>
+  </si>
+  <si>
+    <t>generation</t>
+  </si>
+  <si>
+    <t>AL45 founded</t>
   </si>
 </sst>
 </file>
@@ -94,7 +97,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -125,9 +128,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -462,137 +466,144 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECEA5D20-3B5F-4E4E-B911-FD5C2BFBFF83}">
-  <dimension ref="B1:D14"/>
+  <dimension ref="B1:E14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="3" width="10.83203125" style="1"/>
-    <col min="4" max="4" width="32.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" style="2"/>
+    <col min="5" max="5" width="32.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B2" s="1">
         <v>29830</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B3" s="1">
         <v>35224</v>
       </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B4" s="1">
         <v>35662</v>
       </c>
-      <c r="D4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B5" s="1">
         <v>35799</v>
       </c>
-      <c r="D5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B6" s="1">
         <v>37503</v>
       </c>
       <c r="C6" s="1">
         <v>37686</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B7" s="1">
         <v>38021</v>
       </c>
       <c r="C7" s="1">
         <v>38195</v>
       </c>
-      <c r="D7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B8" s="1">
         <v>38377</v>
       </c>
       <c r="C8" s="1">
         <v>38426</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B9" s="1">
         <v>39630</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B10" s="1">
         <v>39995</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B11" s="1">
         <v>40031</v>
       </c>
       <c r="C11" s="1">
         <v>40230</v>
       </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="E11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B12" s="1">
         <v>40483</v>
       </c>
-      <c r="D12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="E12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B13" s="1">
         <v>41456</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="2">
+        <v>615</v>
+      </c>
+      <c r="E13" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B14" s="1">
         <v>41487</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>